<commit_message>
The 'Sync Live from TWS' button now features a bolder font and a slightly darker green background
</commit_message>
<xml_diff>
--- a/convexitydesk/logo/convexitydesk_logo.xlsx
+++ b/convexitydesk/logo/convexitydesk_logo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\donca\Desktop\Desktop HP Envy x360 al 22Abr24\Docs Manuel\IBKR_Options\convexitydesk\logo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A4BAFA-6D15-46D1-A634-20EFCA6B7532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17866F5D-5845-4EED-A877-4552E30B08D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{B8A67C6C-C630-4024-AB74-D96B6D15649F}"/>
   </bookViews>
@@ -56,7 +56,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -93,6 +93,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -130,6 +136,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,10 +674,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C5D5A1B-F6A9-4C9C-B115-C8AA2D3401E2}">
-  <dimension ref="H12:U125"/>
+  <dimension ref="H12:AB125"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="17" width="3.42578125" customWidth="1"/>
+    <col min="6" max="32" width="3.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="12" spans="9:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1125,7 +1132,7 @@
       <c r="M110" s="6"/>
       <c r="N110" s="7"/>
     </row>
-    <row r="118" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H118" s="7"/>
       <c r="I118" s="7"/>
       <c r="J118" s="7"/>
@@ -1134,8 +1141,16 @@
       <c r="M118" s="7"/>
       <c r="N118" s="7"/>
       <c r="O118" s="7"/>
-    </row>
-    <row r="119" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U118" s="8"/>
+      <c r="V118" s="8"/>
+      <c r="W118" s="8"/>
+      <c r="X118" s="8"/>
+      <c r="Y118" s="8"/>
+      <c r="Z118" s="8"/>
+      <c r="AA118" s="8"/>
+      <c r="AB118" s="8"/>
+    </row>
+    <row r="119" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H119" s="7"/>
       <c r="I119" s="7"/>
       <c r="J119" s="6"/>
@@ -1144,8 +1159,16 @@
       <c r="M119" s="7"/>
       <c r="N119" s="7"/>
       <c r="O119" s="7"/>
-    </row>
-    <row r="120" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U119" s="8"/>
+      <c r="V119" s="8"/>
+      <c r="W119" s="6"/>
+      <c r="X119" s="6"/>
+      <c r="Y119" s="8"/>
+      <c r="Z119" s="8"/>
+      <c r="AA119" s="8"/>
+      <c r="AB119" s="8"/>
+    </row>
+    <row r="120" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H120" s="7"/>
       <c r="I120" s="6"/>
       <c r="J120" s="7"/>
@@ -1154,8 +1177,16 @@
       <c r="M120" s="7"/>
       <c r="N120" s="7"/>
       <c r="O120" s="7"/>
-    </row>
-    <row r="121" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U120" s="8"/>
+      <c r="V120" s="6"/>
+      <c r="W120" s="8"/>
+      <c r="X120" s="8"/>
+      <c r="Y120" s="8"/>
+      <c r="Z120" s="8"/>
+      <c r="AA120" s="8"/>
+      <c r="AB120" s="8"/>
+    </row>
+    <row r="121" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H121" s="7"/>
       <c r="I121" s="7"/>
       <c r="J121" s="6"/>
@@ -1164,8 +1195,16 @@
       <c r="M121" s="7"/>
       <c r="N121" s="7"/>
       <c r="O121" s="7"/>
-    </row>
-    <row r="122" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U121" s="8"/>
+      <c r="V121" s="8"/>
+      <c r="W121" s="6"/>
+      <c r="X121" s="6"/>
+      <c r="Y121" s="8"/>
+      <c r="Z121" s="8"/>
+      <c r="AA121" s="8"/>
+      <c r="AB121" s="8"/>
+    </row>
+    <row r="122" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H122" s="7"/>
       <c r="I122" s="7"/>
       <c r="J122" s="7"/>
@@ -1174,8 +1213,16 @@
       <c r="M122" s="6"/>
       <c r="N122" s="7"/>
       <c r="O122" s="7"/>
-    </row>
-    <row r="123" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U122" s="8"/>
+      <c r="V122" s="8"/>
+      <c r="W122" s="8"/>
+      <c r="X122" s="8"/>
+      <c r="Y122" s="6"/>
+      <c r="Z122" s="6"/>
+      <c r="AA122" s="8"/>
+      <c r="AB122" s="8"/>
+    </row>
+    <row r="123" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H123" s="7"/>
       <c r="I123" s="7"/>
       <c r="J123" s="7"/>
@@ -1184,8 +1231,16 @@
       <c r="M123" s="7"/>
       <c r="N123" s="6"/>
       <c r="O123" s="7"/>
-    </row>
-    <row r="124" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U123" s="8"/>
+      <c r="V123" s="8"/>
+      <c r="W123" s="8"/>
+      <c r="X123" s="8"/>
+      <c r="Y123" s="6"/>
+      <c r="Z123" s="8"/>
+      <c r="AA123" s="6"/>
+      <c r="AB123" s="8"/>
+    </row>
+    <row r="124" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H124" s="7"/>
       <c r="I124" s="7"/>
       <c r="J124" s="7"/>
@@ -1194,8 +1249,16 @@
       <c r="M124" s="6"/>
       <c r="N124" s="7"/>
       <c r="O124" s="7"/>
-    </row>
-    <row r="125" spans="8:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U124" s="8"/>
+      <c r="V124" s="8"/>
+      <c r="W124" s="8"/>
+      <c r="X124" s="8"/>
+      <c r="Y124" s="6"/>
+      <c r="Z124" s="6"/>
+      <c r="AA124" s="8"/>
+      <c r="AB124" s="8"/>
+    </row>
+    <row r="125" spans="8:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H125" s="7"/>
       <c r="I125" s="7"/>
       <c r="J125" s="7"/>
@@ -1204,6 +1267,14 @@
       <c r="M125" s="7"/>
       <c r="N125" s="7"/>
       <c r="O125" s="7"/>
+      <c r="U125" s="8"/>
+      <c r="V125" s="8"/>
+      <c r="W125" s="8"/>
+      <c r="X125" s="8"/>
+      <c r="Y125" s="8"/>
+      <c r="Z125" s="8"/>
+      <c r="AA125" s="8"/>
+      <c r="AB125" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>